<commit_message>
Update device report description
</commit_message>
<xml_diff>
--- a/api/templates/device_report/en.xlsx
+++ b/api/templates/device_report/en.xlsx
@@ -37,7 +37,7 @@
     <t xml:space="preserve">&lt;SitesLabel&gt;: &lt;Sites&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">Please note that this report includes MTB/Rif as well as MTB ULTRA results</t>
+    <t xml:space="preserve">Please note that this report includes MTB/Rif, MTB ULTRA and MTB XDR results</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;Table&gt;</t>
@@ -457,7 +457,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Y14"/>
-  <sheetFormatPr defaultColWidth="11.15625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.17578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="30.58"/>

</xml_diff>

<commit_message>
Add MTB+ and MTB Trace Detected columns in Device Report
</commit_message>
<xml_diff>
--- a/api/templates/device_report/en.xlsx
+++ b/api/templates/device_report/en.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t xml:space="preserve">GeneXpert Devices</t>
   </si>
@@ -46,7 +46,7 @@
     <t xml:space="preserve">Device</t>
   </si>
   <si>
-    <t xml:space="preserve">Site Name</t>
+    <t xml:space="preserve">Site name</t>
   </si>
   <si>
     <t xml:space="preserve">State</t>
@@ -61,24 +61,28 @@
     <t xml:space="preserve"># MTB-</t>
   </si>
   <si>
-    <t xml:space="preserve"># MTB+ RIF
-sens</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># MTB+ RIF
-res</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># MTB+ RIF indeterminate</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># error results</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># invalid results</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># no result</t>
+    <t xml:space="preserve"># MTB+</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># MTB Trace Detected</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># MTB Error</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># MTB Invalid</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># MTB No Result</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># Rif Not Detected</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># Rif Detected</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># Rif Indeterminate</t>
   </si>
   <si>
     <t xml:space="preserve"># INH</t>
@@ -99,12 +103,10 @@
     <t xml:space="preserve"># ETH</t>
   </si>
   <si>
-    <t xml:space="preserve"># Xpert
-modules in use</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No of days
-interrupted service</t>
+    <t xml:space="preserve"># Modules in use</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># Days of interrupted service</t>
   </si>
   <si>
     <t xml:space="preserve">Reason for interruption</t>
@@ -113,13 +115,13 @@
     <t xml:space="preserve">Error rate</t>
   </si>
   <si>
-    <t xml:space="preserve">Error/Invalid Rate</t>
+    <t xml:space="preserve">Error/Invalid rate</t>
   </si>
   <si>
     <t xml:space="preserve">Comment</t>
   </si>
   <si>
-    <t xml:space="preserve"># total Xpert tests</t>
+    <t xml:space="preserve"># Total tests</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;name&gt;</t>
@@ -140,6 +142,21 @@
     <t xml:space="preserve">&lt;totalMtbNegative&gt;</t>
   </si>
   <si>
+    <t xml:space="preserve">&lt;totalMtbDetected&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;totalMtbTraceDetected&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;totalErrors&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;mtbInvalid&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;mtbNoResult&gt;</t>
+  </si>
+  <si>
     <t xml:space="preserve">&lt;totalMtbSens&gt;</t>
   </si>
   <si>
@@ -147,15 +164,6 @@
   </si>
   <si>
     <t xml:space="preserve">&lt;totalMtbIndeterminate&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;totalErrors&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;mtbInvalid&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;mtbNoResult&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;INH&gt;</t>
@@ -197,7 +205,7 @@
     <numFmt numFmtId="165" formatCode="0.00%"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ hh:mm"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -238,6 +246,14 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <i val="true"/>
       <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -314,7 +330,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -347,15 +363,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -375,7 +399,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -456,20 +480,21 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Y14"/>
-  <sheetFormatPr defaultColWidth="11.17578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AMJ14"/>
+  <sheetFormatPr defaultColWidth="11.21484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="30.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="11.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="9" style="0" width="15.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="13.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="13" style="0" width="15.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="20" style="0" width="20.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="22" style="1" width="20.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="33.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="20.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="15.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="11.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="14" style="0" width="15.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="22" style="0" width="20.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="24" style="1" width="20.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="33.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="20.57"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -513,7 +538,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" s="10" customFormat="true" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" s="12" customFormat="true" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
         <v>7</v>
       </c>
@@ -532,25 +557,25 @@
       <c r="F10" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="7" t="s">
         <v>14</v>
       </c>
       <c r="I10" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="J10" s="7" t="s">
+      <c r="J10" s="8" t="s">
         <v>16</v>
       </c>
       <c r="K10" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="L10" s="7" t="s">
+      <c r="L10" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="M10" s="7" t="s">
+      <c r="M10" s="10" t="s">
         <v>19</v>
       </c>
       <c r="N10" s="7" t="s">
@@ -568,113 +593,128 @@
       <c r="R10" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="S10" s="8" t="s">
+      <c r="S10" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="T10" s="8" t="s">
+      <c r="T10" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="U10" s="7" t="s">
+      <c r="U10" s="9" t="s">
         <v>27</v>
       </c>
       <c r="V10" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="W10" s="9" t="s">
+      <c r="W10" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="X10" s="7" t="s">
+      <c r="X10" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="Y10" s="7" t="s">
+      <c r="Y10" s="11" t="s">
         <v>31</v>
       </c>
+      <c r="Z10" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="AA10" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="AMH10" s="0"/>
+      <c r="AMI10" s="0"/>
+      <c r="AMJ10" s="0"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" s="11" t="s">
+      <c r="A11" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="B11" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="C11" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="D11" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="E11" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="H11" s="11" t="s">
+      <c r="F11" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="I11" s="11" t="s">
+      <c r="G11" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="J11" s="12" t="s">
+      <c r="H11" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="K11" s="12" t="s">
+      <c r="I11" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="L11" s="12" t="s">
+      <c r="J11" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="M11" s="12" t="s">
+      <c r="K11" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="N11" s="12" t="s">
+      <c r="L11" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="O11" s="12" t="s">
+      <c r="M11" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="P11" s="12" t="s">
+      <c r="N11" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="Q11" s="12" t="s">
+      <c r="O11" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="R11" s="12" t="s">
+      <c r="P11" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="S11" s="11" t="s">
+      <c r="Q11" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="T11" s="11" t="s">
+      <c r="R11" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="U11" s="11" t="s">
+      <c r="S11" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="V11" s="13" t="e">
-        <f aca="false">IF(Y11=0,0,J11/Y11)</f>
+      <c r="T11" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="U11" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="V11" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="W11" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="X11" s="15" t="e">
+        <f aca="false">IF(AA11=0,0,I11/AA11)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="W11" s="14" t="e">
-        <f aca="false">IF(Y11=0,0,(J11+K11)/Y11)</f>
+      <c r="Y11" s="16" t="e">
+        <f aca="false">IF(AA11=0,0,(I11+J11)/AA11)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="X11" s="14" t="e">
-        <f aca="false">IF(W11&gt;0.05,"High Rate of Errors/Invalids. Contact Lab.","")</f>
+      <c r="Z11" s="16" t="e">
+        <f aca="false">IF(Y11&gt;0.05,"High Rate of Errors/Invalids. Contact Lab.","")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="Y11" s="11" t="s">
-        <v>53</v>
+      <c r="AA11" s="13" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Add descriptions inside device report templates
</commit_message>
<xml_diff>
--- a/api/templates/device_report/en.xlsx
+++ b/api/templates/device_report/en.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="61">
   <si>
     <t xml:space="preserve">GeneXpert Devices</t>
   </si>
@@ -28,16 +28,28 @@
     <t xml:space="preserve">Dates: &lt;Dates&gt;</t>
   </si>
   <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
     <t xml:space="preserve">&lt;StatesLabel&gt;: &lt;States&gt;</t>
   </si>
   <si>
+    <t xml:space="preserve">Please note that this report includes MTB/Rif, MTB ULTRA and MTB XDR results</t>
+  </si>
+  <si>
     <t xml:space="preserve">&lt;LgasLabel&gt;: &lt;Lgas&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;SitesLabel&gt;: &lt;Sites&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">Please note that this report includes MTB/Rif, MTB ULTRA and MTB XDR results</t>
+    <t xml:space="preserve">References</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># Days of interrupted service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Counts the number of days when a device was at least once reported with any of the inactivity statuses (including also the statuses Unknown and No Tests Performed)</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;Table&gt;</t>
@@ -103,10 +115,7 @@
     <t xml:space="preserve"># ETH</t>
   </si>
   <si>
-    <t xml:space="preserve"># Modules in use</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># Days of interrupted service</t>
+    <t xml:space="preserve"># Modules used in the date range</t>
   </si>
   <si>
     <t xml:space="preserve">Reason for interruption</t>
@@ -242,18 +251,18 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
       <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
+      <charset val="204"/>
     </font>
     <font>
       <b val="true"/>
-      <i val="true"/>
       <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -330,7 +339,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -345,21 +354,25 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -367,15 +380,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -481,10 +494,12 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AMJ14"/>
-  <sheetFormatPr defaultColWidth="11.21484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.30859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="30.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="35.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="33.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="11.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="15.57"/>
@@ -509,214 +524,233 @@
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C2" s="0" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>2</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="50.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
-        <v>5</v>
-      </c>
+      <c r="A5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="83.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6"/>
+      <c r="A8" s="8"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" s="12" customFormat="true" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" s="13" customFormat="true" ht="50.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="J10" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="K10" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="L10" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="M10" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="N10" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="O10" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="P10" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q10" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="R10" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="S10" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="T10" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="U10" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="V10" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="K10" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="L10" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="M10" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="N10" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O10" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="P10" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q10" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="R10" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="S10" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="T10" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="U10" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="V10" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="X10" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="Y10" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="Z10" s="7" t="s">
+      <c r="W10" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="AA10" s="7" t="s">
+      <c r="X10" s="12" t="s">
         <v>33</v>
+      </c>
+      <c r="Y10" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z10" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA10" s="9" t="s">
+        <v>36</v>
       </c>
       <c r="AMH10" s="0"/>
       <c r="AMI10" s="0"/>
       <c r="AMJ10" s="0"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" s="13" t="s">
+      <c r="A11" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="B11" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="C11" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G11" s="13" t="s">
+      <c r="D11" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="E11" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="I11" s="14" t="s">
+      <c r="F11" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="J11" s="14" t="s">
+      <c r="G11" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="K11" s="14" t="s">
+      <c r="H11" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="L11" s="13" t="s">
+      <c r="I11" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="M11" s="13" t="s">
+      <c r="J11" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="N11" s="13" t="s">
+      <c r="K11" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="O11" s="14" t="s">
+      <c r="L11" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="P11" s="14" t="s">
+      <c r="M11" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="Q11" s="14" t="s">
+      <c r="N11" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="R11" s="14" t="s">
+      <c r="O11" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="S11" s="14" t="s">
+      <c r="P11" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="T11" s="14" t="s">
+      <c r="Q11" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="U11" s="13" t="s">
+      <c r="R11" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="V11" s="13" t="s">
+      <c r="S11" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="W11" s="13" t="s">
+      <c r="T11" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="X11" s="15" t="e">
+      <c r="U11" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="V11" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="W11" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="X11" s="16" t="e">
         <f aca="false">IF(AA11=0,0,I11/AA11)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="Y11" s="16" t="e">
+      <c r="Y11" s="17" t="e">
         <f aca="false">IF(AA11=0,0,(I11+J11)/AA11)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="Z11" s="16" t="e">
+      <c r="Z11" s="17" t="e">
         <f aca="false">IF(Y11&gt;0.05,"High Rate of Errors/Invalids. Contact Lab.","")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AA11" s="13" t="s">
-        <v>57</v>
+      <c r="AA11" s="14" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C3:D3"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>